<commit_message>
feat: adiciona opcao de excluir e ajustes de usabilidade
</commit_message>
<xml_diff>
--- a/Formulário Pedido Orçamento.xlsx
+++ b/Formulário Pedido Orçamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PenDrivers\ProjetosCursor\SiteGigaeletro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ACC29008-793A-46FF-989B-C75FCA72BA12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C726335-69D6-4C8E-B37F-B442568DA012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="12240" xr2:uid="{819BF0D0-E312-4163-846A-FF994743DCDD}"/>
   </bookViews>
@@ -25,15 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
   <si>
     <t>Nome:</t>
   </si>
   <si>
     <t>CPF/CNPJ:</t>
-  </si>
-  <si>
-    <t>Celular:</t>
   </si>
   <si>
     <t>End:</t>
@@ -98,6 +95,12 @@
       </rPr>
       <t>O PRAZO DE VALIDADE DESTE ORÇAMENTO É DE 15 (QUINZE) DIAS A CONTAR DA DATA DO SEU ENVIO.</t>
     </r>
+  </si>
+  <si>
+    <t>Telefone / Celular:</t>
+  </si>
+  <si>
+    <t>e-mail:</t>
   </si>
 </sst>
 </file>
@@ -166,7 +169,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -177,17 +180,6 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top/>
       <bottom style="medium">
         <color indexed="64"/>
@@ -218,7 +210,18 @@
       </left>
       <right/>
       <top/>
-      <bottom style="thin">
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -226,14 +229,44 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="thin">
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -248,7 +281,7 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -257,25 +290,21 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -286,7 +315,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -299,7 +328,7 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -308,47 +337,68 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -366,55 +416,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>106680</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>7621</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>777240</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>22861</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagem 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F1888503-E44A-40A5-F001-B05515A83D14}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="106680" y="464821"/>
-          <a:ext cx="7010400" cy="3688080"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -714,199 +715,220 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E9DD685-733C-4B3E-9840-D300CE180D27}">
-  <dimension ref="J2:R18"/>
+  <dimension ref="B2:L18"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="L2" s="9" t="s">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="D2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+    </row>
+    <row r="3" spans="2:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B4" s="2"/>
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B5" s="2"/>
+      <c r="C5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="I5" s="4"/>
+      <c r="J5" s="3"/>
+    </row>
+    <row r="6" spans="2:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="2"/>
+      <c r="C6" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6" s="12"/>
+      <c r="J6" s="3"/>
+    </row>
+    <row r="7" spans="2:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="2"/>
+      <c r="C7" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I7" s="12"/>
+      <c r="J7" s="3"/>
+    </row>
+    <row r="8" spans="2:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+    </row>
+    <row r="9" spans="2:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B9" s="2"/>
+      <c r="C9" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="I9" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" s="3"/>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B10" s="2"/>
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B11" s="2"/>
+      <c r="J11" s="3"/>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B12" s="2"/>
+      <c r="J12" s="3"/>
+      <c r="L12" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B13" s="2"/>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="B14" s="2"/>
+      <c r="J14" s="3"/>
+      <c r="L14" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B15" s="2"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="3"/>
+    </row>
+    <row r="16" spans="2:12" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="20"/>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
+      <c r="B17" s="2"/>
+      <c r="C17" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-    </row>
-    <row r="3" spans="10:18" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
-    </row>
-    <row r="4" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J4" s="2"/>
-      <c r="K4" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="L4" s="10"/>
-      <c r="M4" s="10"/>
-      <c r="N4" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="O4" s="10"/>
-      <c r="P4" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q4" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="R4" s="3"/>
-    </row>
-    <row r="5" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J5" s="2"/>
-      <c r="K5" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="L5" s="10"/>
-      <c r="M5" s="10"/>
-      <c r="N5" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="O5" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="P5" s="10"/>
-      <c r="Q5" s="10"/>
-      <c r="R5" s="3"/>
-    </row>
-    <row r="6" spans="10:18" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="J6" s="2"/>
-      <c r="K6" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="O6" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="3"/>
-    </row>
-    <row r="7" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="K7" s="12"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="12"/>
-      <c r="N7" s="12"/>
-      <c r="O7" s="12"/>
-      <c r="P7" s="12"/>
-      <c r="Q7" s="12"/>
-    </row>
-    <row r="8" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J8" s="2"/>
-      <c r="K8" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="L8" s="19" t="s">
-        <v>10</v>
-      </c>
-      <c r="M8" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="N8" s="19"/>
-      <c r="O8" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="P8" s="19" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q8" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="R8" s="3"/>
-    </row>
-    <row r="9" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J9" s="2"/>
-      <c r="R9" s="3"/>
-    </row>
-    <row r="10" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J10" s="2"/>
-      <c r="R10" s="3"/>
-    </row>
-    <row r="11" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J11" s="2"/>
-      <c r="R11" s="3"/>
-    </row>
-    <row r="12" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J12" s="2"/>
-      <c r="R12" s="3"/>
-    </row>
-    <row r="13" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J13" s="2"/>
-      <c r="R13" s="3"/>
-    </row>
-    <row r="14" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J14" s="2"/>
-      <c r="K14" s="4"/>
-      <c r="L14" s="5"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
-      <c r="P14" s="5"/>
-      <c r="Q14" s="6"/>
-      <c r="R14" s="3"/>
-    </row>
-    <row r="15" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-      <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="7"/>
-      <c r="Q15" s="7"/>
-    </row>
-    <row r="16" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J16" s="2"/>
-      <c r="K16" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="14"/>
-      <c r="P16" s="18" t="s">
+      <c r="I17" s="19"/>
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" spans="2:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B18" s="2"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="Q16" s="18"/>
-      <c r="R16" s="3"/>
-    </row>
-    <row r="17" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J17" s="2"/>
-      <c r="K17" s="16"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q17" s="21"/>
-      <c r="R17" s="3"/>
-    </row>
-    <row r="18" spans="10:18" x14ac:dyDescent="0.35">
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
-      <c r="N18" s="15"/>
-      <c r="O18" s="15"/>
-      <c r="P18" s="15"/>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="15"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="L2:P2"/>
-    <mergeCell ref="K16:O17"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="D2:H2"/>
+    <mergeCell ref="C17:G18"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="H18:I18"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>